<commit_message>
model sonuc graph calismasi
</commit_message>
<xml_diff>
--- a/results/assignmentModelSummary.xlsx
+++ b/results/assignmentModelSummary.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10511"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/begumyilmaz/Documents/okul/koç/4.2/bitirme/bitirmeRepoYeni/indr491/results/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C850B31-9F32-4648-9E56-F020A19DA797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -46,29 +40,29 @@
     <t>Hammadde kullanımı</t>
   </si>
   <si>
-    <t>Toplam stok: 11677.100000000006</t>
-  </si>
-  <si>
-    <t>Toplam tahsis: 8355.10908240567</t>
+    <t>Toplam stok: 7195.9800000000005</t>
+  </si>
+  <si>
+    <t>Toplam tahsis: 7195.9800000000005</t>
   </si>
   <si>
     <t>%87.05448007313169</t>
   </si>
   <si>
-    <t>%73.4346771828034</t>
+    <t>%73.43467718280338</t>
   </si>
   <si>
     <t>%2.501453996474222</t>
   </si>
   <si>
-    <t>%71.55123346041111</t>
+    <t>%100.0</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -131,21 +125,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -183,7 +169,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -217,7 +203,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -252,10 +237,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -428,17 +412,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.33203125" customWidth="1"/>
-    <col min="3" max="3" width="17.83203125" customWidth="1"/>
-    <col min="4" max="4" width="19.1640625" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -452,7 +430,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -466,12 +444,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>5</v>
       </c>
       <c r="B3">
-        <v>4564.9210000000003</v>
+        <v>4564.921</v>
       </c>
       <c r="C3">
         <v>3352.235000000001</v>
@@ -480,7 +458,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -494,7 +472,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
         <v>7</v>
       </c>

</xml_diff>